<commit_message>
feat(excel): implement visual interactive Excel mapper with context menu, badges and read_only performance optimizations
</commit_message>
<xml_diff>
--- a/excel/Hodiny2026.xlsx
+++ b/excel/Hodiny2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="MMhod26" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MMcash26" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="08hod25" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="08hod26" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="08cash26" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="01hod25" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMhod26" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMcash26" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08hod25" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08hod26" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08cash26" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01hod25" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6099,7 +6099,7 @@
         <f>MAX(0,H17-8)</f>
         <v/>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="0" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="0">

</xml_diff>

<commit_message>
feat(excel): add cash sheet MMcash26 expensee recording and zalohy integration
</commit_message>
<xml_diff>
--- a/excel/Hodiny2026.xlsx
+++ b/excel/Hodiny2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMhod26" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMcash26" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08hod25" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08hod26" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08cash26" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01hod25" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MMhod26" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MMcash26" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="08hod25" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="08hod26" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="08cash26" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="01hod25" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8146,8 +8146,14 @@
       <c r="N4" s="38" t="n"/>
       <c r="O4" s="37" t="n"/>
       <c r="P4" s="36" t="n"/>
-      <c r="Q4" s="41" t="n"/>
-      <c r="R4" s="42" t="n"/>
+      <c r="Q4" s="41" t="n">
+        <v>500</v>
+      </c>
+      <c r="R4" s="42" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
       <c r="S4" s="41" t="n"/>
       <c r="T4" s="42" t="n"/>
       <c r="U4" s="41" t="n"/>

</xml_diff>

<commit_message>
feat(excel): implement advance column allocation per employee in cash sheets
</commit_message>
<xml_diff>
--- a/excel/Hodiny2026.xlsx
+++ b/excel/Hodiny2026.xlsx
@@ -7956,7 +7956,7 @@
       </c>
       <c r="Q2" s="11" t="inlineStr">
         <is>
-          <t>Sloupec1</t>
+          <t>Čáp</t>
         </is>
       </c>
       <c r="R2" s="12" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="S2" s="13" t="inlineStr">
         <is>
-          <t>Sloupec2</t>
+          <t>Novák</t>
         </is>
       </c>
       <c r="T2" s="12" t="inlineStr">
@@ -8099,8 +8099,14 @@
           <t>20.08.2026</t>
         </is>
       </c>
-      <c r="S3" s="25" t="n"/>
-      <c r="T3" s="26" t="n"/>
+      <c r="S3" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="T3" s="26" t="inlineStr">
+        <is>
+          <t>12.08.2026</t>
+        </is>
+      </c>
       <c r="U3" s="25" t="n"/>
       <c r="V3" s="26" t="n"/>
       <c r="W3" s="27" t="n"/>
@@ -8199,8 +8205,14 @@
       <c r="N5" s="20" t="n"/>
       <c r="O5" s="19" t="n"/>
       <c r="P5" s="18" t="n"/>
-      <c r="Q5" s="25" t="n"/>
-      <c r="R5" s="26" t="n"/>
+      <c r="Q5" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" s="26" t="inlineStr">
+        <is>
+          <t>01.08.2026</t>
+        </is>
+      </c>
       <c r="S5" s="25" t="n"/>
       <c r="T5" s="26" t="n"/>
       <c r="U5" s="25" t="n"/>
@@ -8254,8 +8266,14 @@
       <c r="N6" s="38" t="n"/>
       <c r="O6" s="37" t="n"/>
       <c r="P6" s="36" t="n"/>
-      <c r="Q6" s="41" t="n"/>
-      <c r="R6" s="42" t="n"/>
+      <c r="Q6" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="R6" s="42" t="inlineStr">
+        <is>
+          <t>10.08.2026</t>
+        </is>
+      </c>
       <c r="S6" s="41" t="n"/>
       <c r="T6" s="42" t="n"/>
       <c r="U6" s="41" t="n"/>

</xml_diff>

<commit_message>
feat(excel): write advances for Čáp into O4+ (EUR) and P4+ (CZK)
</commit_message>
<xml_diff>
--- a/excel/Hodiny2026.xlsx
+++ b/excel/Hodiny2026.xlsx
@@ -8150,8 +8150,12 @@
       <c r="L4" s="39" t="n"/>
       <c r="M4" s="40" t="n"/>
       <c r="N4" s="38" t="n"/>
-      <c r="O4" s="37" t="n"/>
-      <c r="P4" s="36" t="n"/>
+      <c r="O4" s="37" t="n">
+        <v>200</v>
+      </c>
+      <c r="P4" s="36" t="n">
+        <v>5000</v>
+      </c>
       <c r="Q4" s="41" t="n">
         <v>500</v>
       </c>
@@ -8203,7 +8207,9 @@
       <c r="L5" s="21" t="n"/>
       <c r="M5" s="22" t="n"/>
       <c r="N5" s="20" t="n"/>
-      <c r="O5" s="19" t="n"/>
+      <c r="O5" s="19" t="n">
+        <v>150</v>
+      </c>
       <c r="P5" s="18" t="n"/>
       <c r="Q5" s="25" t="n">
         <v>100</v>

</xml_diff>